<commit_message>
Figures and analyses for the additional genes
</commit_message>
<xml_diff>
--- a/datasets/All data combined.xlsx
+++ b/datasets/All data combined.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucia\OneDrive - Wageningen University &amp; Research\UCI_projects\Project_8 (Reviews)\Family\Pere\doctorado\datasets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wageningenur4-my.sharepoint.com/personal/luciana_chavezrodriguez_wur_nl/Documents/UCI_projects/Project_8 (Reviews)/Family/Pere/doctorado/datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C8CB1C-E085-459C-911F-489FBB0B6CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{D1C8CB1C-E085-459C-911F-489FBB0B6CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48B7CFEA-252F-4B57-BC14-7FDBAA4E3518}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{4666BC1F-E1FD-498B-BFD1-D32BBF6EE224}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{4666BC1F-E1FD-498B-BFD1-D32BBF6EE224}"/>
   </bookViews>
   <sheets>
     <sheet name="LLM1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="Thesis" sheetId="7" r:id="rId4"/>
     <sheet name="MET1" sheetId="4" r:id="rId5"/>
     <sheet name="CTZ1" sheetId="5" r:id="rId6"/>
-    <sheet name="YAL1" sheetId="6" r:id="rId7"/>
+    <sheet name="Thesis_2" sheetId="8" r:id="rId7"/>
+    <sheet name="YAL1" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029" iterateCount="1"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="36">
   <si>
     <t>SXM</t>
   </si>
@@ -27265,6 +27266,1869 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E119322-35AE-4E68-9B45-080479264335}">
+  <dimension ref="A1:E109"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="5">
+        <v>1</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="6">
+        <v>48.864362006586802</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="7">
+        <v>14.843353960678201</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="7">
+        <v>70.7341918064634</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="6">
+        <v>3.3244154026341501</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="7">
+        <v>2.6246176118321101</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="7">
+        <v>3.4840629764618898</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="6">
+        <v>2.5482771356981599</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="7">
+        <v>1.65657427183926</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="7">
+        <v>0.994818515081486</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="5">
+        <v>1</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="5">
+        <v>1</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="5">
+        <v>1</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="6">
+        <v>3.3501456436288102</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="6">
+        <v>2.23969607490459</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="6">
+        <v>4.7321795162719198</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1.71247483982947</v>
+      </c>
+      <c r="D20" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="6">
+        <v>1.3979890879977801</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.87979056890749596</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="6">
+        <v>1.8782721145427199</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="6">
+        <v>2.2721124032753202</v>
+      </c>
+      <c r="D24" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="6">
+        <v>2.1223775559717599</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="5">
+        <v>1</v>
+      </c>
+      <c r="D26" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="5">
+        <v>1</v>
+      </c>
+      <c r="D27" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="5">
+        <v>1</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="6">
+        <v>15.511725995950799</v>
+      </c>
+      <c r="D29" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="6">
+        <v>15.707852860823101</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="6">
+        <v>10.632618410004399</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="6">
+        <v>0.50462087704057301</v>
+      </c>
+      <c r="D32" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E32">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="6">
+        <v>0.300353013279754</v>
+      </c>
+      <c r="D33" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="6">
+        <v>0.65182691797723102</v>
+      </c>
+      <c r="D34" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="6">
+        <v>1.5335294301467699</v>
+      </c>
+      <c r="D35" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>29</v>
+      </c>
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="6">
+        <v>1.2313250186186</v>
+      </c>
+      <c r="D36" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>29</v>
+      </c>
+      <c r="B37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" s="6">
+        <v>2.1114805564358301</v>
+      </c>
+      <c r="D37" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" t="s">
+        <v>21</v>
+      </c>
+      <c r="C38" s="5">
+        <v>1</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" s="5">
+        <v>1</v>
+      </c>
+      <c r="D39" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" s="5">
+        <v>1</v>
+      </c>
+      <c r="D40" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>0</v>
+      </c>
+      <c r="B41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" s="6">
+        <v>0.17354668044379701</v>
+      </c>
+      <c r="D41" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B42" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" s="6">
+        <v>0.18059602292267499</v>
+      </c>
+      <c r="D42" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>0</v>
+      </c>
+      <c r="B43" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" s="6">
+        <v>0.24323697470759401</v>
+      </c>
+      <c r="D43" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>0</v>
+      </c>
+      <c r="B44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44" s="6">
+        <v>2.7105488211786999</v>
+      </c>
+      <c r="D44" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" s="6">
+        <v>1.3807982983170899</v>
+      </c>
+      <c r="D45" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>0</v>
+      </c>
+      <c r="B46" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" s="6">
+        <v>1.26217132371539</v>
+      </c>
+      <c r="D46" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>0</v>
+      </c>
+      <c r="B47" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" s="6">
+        <v>1.1707018304564001</v>
+      </c>
+      <c r="D47" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E47">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>0</v>
+      </c>
+      <c r="B48" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" s="6">
+        <v>0.91568600308244597</v>
+      </c>
+      <c r="D48" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E48">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" t="s">
+        <v>21</v>
+      </c>
+      <c r="C49" s="6">
+        <v>2.4059651971443099</v>
+      </c>
+      <c r="D49" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E49">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>9</v>
+      </c>
+      <c r="B50" t="s">
+        <v>21</v>
+      </c>
+      <c r="C50" s="5">
+        <v>1</v>
+      </c>
+      <c r="D50" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>9</v>
+      </c>
+      <c r="B51" t="s">
+        <v>21</v>
+      </c>
+      <c r="C51" s="5">
+        <v>1</v>
+      </c>
+      <c r="D51" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52" t="s">
+        <v>21</v>
+      </c>
+      <c r="C52" s="5">
+        <v>1</v>
+      </c>
+      <c r="D52" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>9</v>
+      </c>
+      <c r="B53" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" s="6">
+        <v>0.39458197786253002</v>
+      </c>
+      <c r="D53" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>9</v>
+      </c>
+      <c r="B54" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54" s="6">
+        <v>0.24271655646683299</v>
+      </c>
+      <c r="D54" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>9</v>
+      </c>
+      <c r="B55" t="s">
+        <v>21</v>
+      </c>
+      <c r="C55" s="6">
+        <v>0.37848063804103299</v>
+      </c>
+      <c r="D55" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>9</v>
+      </c>
+      <c r="B56" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56" s="6">
+        <v>0.35288586100513503</v>
+      </c>
+      <c r="D56" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E56">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>9</v>
+      </c>
+      <c r="B57" t="s">
+        <v>21</v>
+      </c>
+      <c r="C57" s="6">
+        <v>0.35266151901595899</v>
+      </c>
+      <c r="D57" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E57">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>9</v>
+      </c>
+      <c r="B58" t="s">
+        <v>21</v>
+      </c>
+      <c r="C58" s="6">
+        <v>0.31149220769074398</v>
+      </c>
+      <c r="D58" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E58">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>9</v>
+      </c>
+      <c r="B59" t="s">
+        <v>21</v>
+      </c>
+      <c r="C59" s="6">
+        <v>1.0565498890582501</v>
+      </c>
+      <c r="D59" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E59">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>9</v>
+      </c>
+      <c r="B60" t="s">
+        <v>21</v>
+      </c>
+      <c r="C60" s="6">
+        <v>0.16503190109615701</v>
+      </c>
+      <c r="D60" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E60">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>9</v>
+      </c>
+      <c r="B61" t="s">
+        <v>21</v>
+      </c>
+      <c r="C61" s="6">
+        <v>0.36715348753020799</v>
+      </c>
+      <c r="D61" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E61">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>29</v>
+      </c>
+      <c r="B62" t="s">
+        <v>21</v>
+      </c>
+      <c r="C62" s="5">
+        <v>1</v>
+      </c>
+      <c r="D62" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>29</v>
+      </c>
+      <c r="B63" t="s">
+        <v>21</v>
+      </c>
+      <c r="C63" s="5">
+        <v>1</v>
+      </c>
+      <c r="D63" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>29</v>
+      </c>
+      <c r="B64" t="s">
+        <v>21</v>
+      </c>
+      <c r="C64" s="5">
+        <v>1</v>
+      </c>
+      <c r="D64" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>29</v>
+      </c>
+      <c r="B65" t="s">
+        <v>21</v>
+      </c>
+      <c r="C65" s="6">
+        <v>0.63487595326824597</v>
+      </c>
+      <c r="D65" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>29</v>
+      </c>
+      <c r="B66" t="s">
+        <v>21</v>
+      </c>
+      <c r="C66" s="6">
+        <v>0.61367601406778605</v>
+      </c>
+      <c r="D66" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>29</v>
+      </c>
+      <c r="B67" t="s">
+        <v>21</v>
+      </c>
+      <c r="C67" s="6">
+        <v>0.61973964725860198</v>
+      </c>
+      <c r="D67" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>29</v>
+      </c>
+      <c r="B68" t="s">
+        <v>21</v>
+      </c>
+      <c r="C68" s="6">
+        <v>0.61332019785104896</v>
+      </c>
+      <c r="D68" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E68">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>29</v>
+      </c>
+      <c r="B69" t="s">
+        <v>21</v>
+      </c>
+      <c r="C69" s="6">
+        <v>0.72583519253423701</v>
+      </c>
+      <c r="D69" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E69">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>29</v>
+      </c>
+      <c r="B70" t="s">
+        <v>21</v>
+      </c>
+      <c r="C70" s="6">
+        <v>0.60170404682206002</v>
+      </c>
+      <c r="D70" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E70">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>29</v>
+      </c>
+      <c r="B71" t="s">
+        <v>21</v>
+      </c>
+      <c r="C71" s="6">
+        <v>1.0457765716071401</v>
+      </c>
+      <c r="D71" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E71">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>29</v>
+      </c>
+      <c r="B72" t="s">
+        <v>21</v>
+      </c>
+      <c r="C72" s="6">
+        <v>1.0009959408378799</v>
+      </c>
+      <c r="D72" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E72">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>29</v>
+      </c>
+      <c r="B73" t="s">
+        <v>21</v>
+      </c>
+      <c r="C73" s="6">
+        <v>1.53522021174533</v>
+      </c>
+      <c r="D73" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E73">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>0</v>
+      </c>
+      <c r="B74" t="s">
+        <v>20</v>
+      </c>
+      <c r="C74" s="5">
+        <v>1</v>
+      </c>
+      <c r="D74" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>0</v>
+      </c>
+      <c r="B75" t="s">
+        <v>20</v>
+      </c>
+      <c r="C75" s="5">
+        <v>1</v>
+      </c>
+      <c r="D75" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" t="s">
+        <v>20</v>
+      </c>
+      <c r="C76" s="5">
+        <v>1</v>
+      </c>
+      <c r="D76" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>0</v>
+      </c>
+      <c r="B77" t="s">
+        <v>20</v>
+      </c>
+      <c r="C77" s="6">
+        <v>0.77328576621947498</v>
+      </c>
+      <c r="D77" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" t="s">
+        <v>20</v>
+      </c>
+      <c r="C78" s="6">
+        <v>0.79490801590326798</v>
+      </c>
+      <c r="D78" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>0</v>
+      </c>
+      <c r="B79" t="s">
+        <v>20</v>
+      </c>
+      <c r="C79" s="6">
+        <v>0.47228729798443903</v>
+      </c>
+      <c r="D79" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>0</v>
+      </c>
+      <c r="B80" t="s">
+        <v>20</v>
+      </c>
+      <c r="C80" s="6">
+        <v>0.55011371315021396</v>
+      </c>
+      <c r="D80" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E80">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>0</v>
+      </c>
+      <c r="B81" t="s">
+        <v>20</v>
+      </c>
+      <c r="C81" s="6">
+        <v>0.74898922082493002</v>
+      </c>
+      <c r="D81" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E81">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>0</v>
+      </c>
+      <c r="B82" t="s">
+        <v>20</v>
+      </c>
+      <c r="C82" s="6">
+        <v>0.49341032047963301</v>
+      </c>
+      <c r="D82" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E82">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>0</v>
+      </c>
+      <c r="B83" t="s">
+        <v>20</v>
+      </c>
+      <c r="C83" s="6">
+        <v>0.86183491495708098</v>
+      </c>
+      <c r="D83" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E83">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>0</v>
+      </c>
+      <c r="B84" t="s">
+        <v>20</v>
+      </c>
+      <c r="C84" s="6">
+        <v>0.41005356663305997</v>
+      </c>
+      <c r="D84" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E84">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B85" t="s">
+        <v>20</v>
+      </c>
+      <c r="C85" s="6">
+        <v>0.83689698650414801</v>
+      </c>
+      <c r="D85" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E85">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>9</v>
+      </c>
+      <c r="B86" t="s">
+        <v>20</v>
+      </c>
+      <c r="C86" s="5">
+        <v>1</v>
+      </c>
+      <c r="D86" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>9</v>
+      </c>
+      <c r="B87" t="s">
+        <v>20</v>
+      </c>
+      <c r="C87" s="5">
+        <v>1</v>
+      </c>
+      <c r="D87" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>9</v>
+      </c>
+      <c r="B88" t="s">
+        <v>20</v>
+      </c>
+      <c r="C88" s="5">
+        <v>1</v>
+      </c>
+      <c r="D88" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>9</v>
+      </c>
+      <c r="B89" t="s">
+        <v>20</v>
+      </c>
+      <c r="C89" s="6">
+        <v>1.2118815021000999</v>
+      </c>
+      <c r="D89" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E89">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>9</v>
+      </c>
+      <c r="B90" t="s">
+        <v>20</v>
+      </c>
+      <c r="C90" s="6">
+        <v>1.5689270613988</v>
+      </c>
+      <c r="D90" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>9</v>
+      </c>
+      <c r="B91" t="s">
+        <v>20</v>
+      </c>
+      <c r="C91" s="6">
+        <v>1.0918440792444299</v>
+      </c>
+      <c r="D91" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>9</v>
+      </c>
+      <c r="B92" t="s">
+        <v>20</v>
+      </c>
+      <c r="C92" s="6">
+        <v>1.76918899802469</v>
+      </c>
+      <c r="D92" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E92">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>9</v>
+      </c>
+      <c r="B93" t="s">
+        <v>20</v>
+      </c>
+      <c r="C93" s="6">
+        <v>2.4265939386561901</v>
+      </c>
+      <c r="D93" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E93">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>9</v>
+      </c>
+      <c r="B94" t="s">
+        <v>20</v>
+      </c>
+      <c r="C94" s="6">
+        <v>1.6327001961469001</v>
+      </c>
+      <c r="D94" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E94">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>9</v>
+      </c>
+      <c r="B95" t="s">
+        <v>20</v>
+      </c>
+      <c r="C95" s="6">
+        <v>0.20300000000000001</v>
+      </c>
+      <c r="D95" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E95">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>9</v>
+      </c>
+      <c r="B96" t="s">
+        <v>20</v>
+      </c>
+      <c r="C96" s="6">
+        <v>0.372185511867347</v>
+      </c>
+      <c r="D96" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E96">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>9</v>
+      </c>
+      <c r="B97" t="s">
+        <v>20</v>
+      </c>
+      <c r="C97" s="6">
+        <v>0.21278867889785399</v>
+      </c>
+      <c r="D97" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E97">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>29</v>
+      </c>
+      <c r="B98" t="s">
+        <v>20</v>
+      </c>
+      <c r="C98" s="5">
+        <v>1</v>
+      </c>
+      <c r="D98" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>29</v>
+      </c>
+      <c r="B99" t="s">
+        <v>20</v>
+      </c>
+      <c r="C99" s="5">
+        <v>1</v>
+      </c>
+      <c r="D99" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>29</v>
+      </c>
+      <c r="B100" t="s">
+        <v>20</v>
+      </c>
+      <c r="C100" s="5">
+        <v>1</v>
+      </c>
+      <c r="D100" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>29</v>
+      </c>
+      <c r="B101" t="s">
+        <v>20</v>
+      </c>
+      <c r="C101" s="6">
+        <v>2.1213631018997501</v>
+      </c>
+      <c r="D101" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E101">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>29</v>
+      </c>
+      <c r="B102" t="s">
+        <v>20</v>
+      </c>
+      <c r="C102" s="6">
+        <v>1.3147042594893801</v>
+      </c>
+      <c r="D102" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>29</v>
+      </c>
+      <c r="B103" t="s">
+        <v>20</v>
+      </c>
+      <c r="C103" s="6">
+        <v>2.0129117754541199</v>
+      </c>
+      <c r="D103" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E103">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>29</v>
+      </c>
+      <c r="B104" t="s">
+        <v>20</v>
+      </c>
+      <c r="C104" s="6">
+        <v>1.96952136195675</v>
+      </c>
+      <c r="D104" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E104">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>29</v>
+      </c>
+      <c r="B105" t="s">
+        <v>20</v>
+      </c>
+      <c r="C105" s="6">
+        <v>2.1593814795211501</v>
+      </c>
+      <c r="D105" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E105">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>29</v>
+      </c>
+      <c r="B106" t="s">
+        <v>20</v>
+      </c>
+      <c r="C106" s="6">
+        <v>1.51613960873232</v>
+      </c>
+      <c r="D106" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E106">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>29</v>
+      </c>
+      <c r="B107" t="s">
+        <v>20</v>
+      </c>
+      <c r="C107" s="6">
+        <v>1.2477779422166799</v>
+      </c>
+      <c r="D107" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E107">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>29</v>
+      </c>
+      <c r="B108" t="s">
+        <v>20</v>
+      </c>
+      <c r="C108" s="6">
+        <v>0.81296581813051605</v>
+      </c>
+      <c r="D108" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E108">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>29</v>
+      </c>
+      <c r="B109" t="s">
+        <v>20</v>
+      </c>
+      <c r="C109" s="6">
+        <v>0.62055871749841196</v>
+      </c>
+      <c r="D109" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="E109">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4625E9-9BE4-428B-8AEB-674C35123233}">
   <dimension ref="B2:T26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>